<commit_message>
Điền phần góp ý minh hoạ và thêm minhhoa.md
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI20K\Day26_Track01_UniPilot\dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI20K\Day26_Track01_TungTungTungSahur\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E20C246-36CD-4234-BD53-F8FF76CFC24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B872F4-7CCD-4DB7-9540-8097BC104287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="0" windowWidth="18660" windowHeight="10488" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="409">
   <si>
     <t>Dashboard Hành Động áp dụng AI — UniPilot (P-127) · v2 — sau kiểm tra chéo</t>
   </si>
@@ -1141,7 +1141,7 @@
     <t>Thay đổi từ v1 → v2 sau kiểm tra chéo</t>
   </si>
   <si>
-    <t>Cột 'Góp ý từ' phải điền tên nhóm phản biện + người góp ý thật sau chặng 3. Đối chiếu với v1/dashboard_hanh_dong_v1.xlsx.</t>
+    <t>Góp ý minh hoạ, viết theo cho phép của trợ giảng: nhóm không có nhóm đối ứng ở chặng 3, nên các thay đổi đến từ tự rà soát theo 4 trục phản biện. Đối chiếu với v1/dashboard_hanh_dong_v1.xlsx.</t>
   </si>
   <si>
     <t>Trục phản biện</t>
@@ -1171,7 +1171,7 @@
     <t>Đây là activity metric: tăng cả khi AI trả lời sai, và đẩy hệ thống trả lời cả câu lẽ ra phải chuyển người.</t>
   </si>
   <si>
-    <t>[Điền: Nhóm phản biện + người góp ý]</t>
+    <t>Minh hoạ: tự rà soát theo trục Chỉ số (Nguyễn Quang Huy)</t>
   </si>
   <si>
     <t>TĐ2</t>
@@ -1189,7 +1189,7 @@
     <t>Baseline v1 gây hiểu lầm: chỉ trả lời 11/20 câu, judge cùng họ Gemini, không phải dữ liệu thật.</t>
   </si>
   <si>
-    <t>[Điền]</t>
+    <t>Minh hoạ: tự rà soát theo trục Chỉ số – bằng chứng (Lê Thị Hoài Thương)</t>
   </si>
   <si>
     <t>TĐ3</t>
@@ -1207,6 +1207,9 @@
     <t>Chẩn đoán Gartner-Lite ra 'Dữ liệu THIẾU' nhưng dashboard v1 không đo → framework chỉ để dán nhãn.</t>
   </si>
   <si>
+    <t>Minh hoạ: tự rà soát theo trục Framework (Nguyễn Thị Minh Khánh)</t>
+  </si>
+  <si>
     <t>TĐ4</t>
   </si>
   <si>
@@ -1222,6 +1225,9 @@
     <t>Không ai biết phải làm gì và ai làm khi chỉ số xấu.</t>
   </si>
   <si>
+    <t>Minh hoạ: tự rà soát theo trục Hành động (Đỗ Lê Việt Anh)</t>
+  </si>
+  <si>
     <t>TĐ5</t>
   </si>
   <si>
@@ -1237,6 +1243,9 @@
     <t>Roadmap không phải cổng quyết định.</t>
   </si>
   <si>
+    <t>Minh hoạ: tự rà soát theo trục Hành động – lộ trình (Lê Thị Châm Anh)</t>
+  </si>
+  <si>
     <t>TĐ6</t>
   </si>
   <si>
@@ -1250,6 +1259,9 @@
   </si>
   <si>
     <t>Tỷ lệ nộp hồ sơ phụ thuộc mùa vụ, không quy được cho AI; CSAT là tự khai, tỷ lệ phản hồi thấp.</t>
+  </si>
+  <si>
+    <t>Minh hoạ: tự rà soát theo trục Chỉ số – giá trị (Lại Bá Quân)</t>
   </si>
   <si>
     <t>Tự kiểm theo yêu cầu nộp bài (§6.4) — tính bằng công thức từ sheet Dashboard</t>
@@ -1745,7 +1757,7 @@
     <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1763,7 +1775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -1771,7 +1783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1803,7 +1815,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
@@ -1811,7 +1823,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -1827,7 +1839,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>20</v>
       </c>
@@ -1846,7 +1858,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -1860,7 +1872,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
@@ -1891,12 +1903,12 @@
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>34</v>
       </c>
@@ -1918,7 +1930,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>39</v>
       </c>
@@ -1935,7 +1947,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>44</v>
       </c>
@@ -1952,7 +1964,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>49</v>
       </c>
@@ -1969,7 +1981,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>54</v>
       </c>
@@ -1986,7 +1998,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>58</v>
       </c>
@@ -2003,7 +2015,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>63</v>
       </c>
@@ -2042,7 +2054,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>71</v>
       </c>
@@ -2059,7 +2071,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>71</v>
       </c>
@@ -2076,7 +2088,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>71</v>
       </c>
@@ -2093,7 +2105,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>81</v>
       </c>
@@ -2110,7 +2122,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>81</v>
       </c>
@@ -2127,7 +2139,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>88</v>
       </c>
@@ -2140,12 +2152,12 @@
       </c>
       <c r="E19" s="4"/>
     </row>
-    <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>92</v>
       </c>
@@ -2162,7 +2174,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>97</v>
       </c>
@@ -2179,7 +2191,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>102</v>
       </c>
@@ -2196,7 +2208,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>107</v>
       </c>
@@ -2213,7 +2225,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>112</v>
       </c>
@@ -2232,7 +2244,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>116</v>
       </c>
@@ -2246,7 +2258,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>120</v>
       </c>
@@ -2260,7 +2272,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>123</v>
       </c>
@@ -2274,7 +2286,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>127</v>
       </c>
@@ -2288,7 +2300,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>130</v>
       </c>
@@ -2319,7 +2331,7 @@
     <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
@@ -2346,7 +2358,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>138</v>
       </c>
@@ -2380,7 +2392,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>146</v>
       </c>
@@ -2397,7 +2409,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>150</v>
       </c>
@@ -2414,7 +2426,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>62</v>
       </c>
@@ -2431,7 +2443,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>158</v>
       </c>
@@ -2448,7 +2460,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>161</v>
       </c>
@@ -2465,7 +2477,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>164</v>
       </c>
@@ -2482,7 +2494,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>169</v>
       </c>
@@ -2499,7 +2511,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>172</v>
       </c>
@@ -2532,7 +2544,7 @@
     <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>177</v>
       </c>
@@ -2556,7 +2568,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>183</v>
       </c>
@@ -2570,7 +2582,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>187</v>
       </c>
@@ -2584,7 +2596,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>191</v>
       </c>
@@ -2615,7 +2627,7 @@
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>195</v>
       </c>
@@ -2637,7 +2649,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>201</v>
       </c>
@@ -2654,7 +2666,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>206</v>
       </c>
@@ -2671,7 +2683,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>211</v>
       </c>
@@ -2712,7 +2724,7 @@
     <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>216</v>
       </c>
@@ -2766,7 +2778,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>231</v>
       </c>
@@ -2810,7 +2822,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>245</v>
       </c>
@@ -2854,7 +2866,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>255</v>
       </c>
@@ -2898,7 +2910,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>266</v>
       </c>
@@ -2942,7 +2954,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>276</v>
       </c>
@@ -2986,7 +2998,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>287</v>
       </c>
@@ -3030,7 +3042,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>298</v>
       </c>
@@ -3074,7 +3086,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>306</v>
       </c>
@@ -3118,7 +3130,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>317</v>
       </c>
@@ -3162,7 +3174,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>326</v>
       </c>
@@ -3206,7 +3218,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>336</v>
       </c>
@@ -3250,7 +3262,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>345</v>
       </c>
@@ -3313,7 +3325,7 @@
     <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
@@ -3343,7 +3355,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>360</v>
       </c>
@@ -3363,7 +3375,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>365</v>
       </c>
@@ -3383,7 +3395,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>371</v>
       </c>
@@ -3400,67 +3412,67 @@
         <v>375</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>370</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -3477,25 +3489,25 @@
     <col min="2" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="B4" s="10">
         <f>COUNTIF(Dashboard!$B$5:$B$16,"Product")</f>
@@ -3507,7 +3519,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTIF(Dashboard!$B$5:$B$16,"Workflow")</f>
@@ -3519,79 +3531,79 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="B6" s="10">
         <f>COUNTBLANK(Dashboard!$G$5:$G$16)</f>
         <v>0</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTBLANK(Dashboard!$H$5:$H$16)</f>
         <v>0</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTBLANK(Dashboard!$I$5:$I$16)</f>
         <v>0</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTBLANK(Dashboard!$K$5:$K$16)</f>
         <v>0</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTBLANK(Dashboard!$M$5:$M$16)</f>
         <v>0</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B11" s="10">
         <f>COUNTIF(Dashboard!$D$5:$D$16,"3*")+COUNTIF(Dashboard!$D$5:$D$16,"4*")+COUNTIF(Dashboard!$D$5:$D$16,"5*")</f>
         <v>11</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="B12" s="10">
         <f>COUNTIF(Dashboard!$N$5:$N$16,"Quyết định")</f>

</xml_diff>

<commit_message>
Xoá phần góp ý minh hoạ, ghi rõ v2 là kết quả tự rà soát
- Xoá minhhoa.md, cột góp ý minh hoạ trong README, memo §3 và sheet 7_Thay_doi_v1_v2
- Ghi chú nhóm không có nhóm đối ứng ở chặng kiểm tra chéo
- Đổi 'sau kiểm tra chéo' thành 'sau tự rà soát' cho nhất quán
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -64,9 +64,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="409">
-  <si>
-    <t>Dashboard Hành Động áp dụng AI — UniPilot (P-127) · v2 — sau kiểm tra chéo</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="402">
+  <si>
+    <t xml:space="preserve">Dashboard Hành Động áp dụng AI — UniPilot (P-127) · v2 — sau tự rà soát</t>
   </si>
   <si>
     <t>Lab Day26 Track01 · Ngày lập: 14/10/2026 · Dữ liệu lấy từ repo P-127; ô 'Đo tuần 1' là số cần thu thập, không phải số giả định.</t>
@@ -727,7 +727,7 @@
     <t>QUY TẮC: MỞ RỘNG (thêm 1 trường) nếu P1, P3, W1 đạt mục tiêu và ≥7/9 chỉ số quyết định đạt · SỬA nếu chất lượng (P1–P4) đạt nhưng quy trình (W1–W4, V1) chưa · DỪNG chủ đề (kill-switch, quay về FAQ tĩnh) nếu QA đúng &lt;80% hoặc ≥2 lỗi nghiêm trọng/tháng.</t>
   </si>
   <si>
-    <t>Dashboard chỉ số · v2 — sau kiểm tra chéo</t>
+    <t xml:space="preserve">Dashboard chỉ số · v2 — sau tự rà soát</t>
   </si>
   <si>
     <t>Đọc từ dưới lên (tầng 1 → 5), ra quyết định dựa trên chỉ số 'Quyết định'. Dòng tô tím = mới/đổi ở v2.</t>
@@ -1138,13 +1138,13 @@
     <t>Bật semantic cache cho chủ đề tự động; rà prompt dài</t>
   </si>
   <si>
-    <t>Thay đổi từ v1 → v2 sau kiểm tra chéo</t>
-  </si>
-  <si>
-    <t>Góp ý minh hoạ, viết theo cho phép của trợ giảng: nhóm không có nhóm đối ứng ở chặng 3, nên các thay đổi đến từ tự rà soát theo 4 trục phản biện. Đối chiếu với v1/dashboard_hanh_dong_v1.xlsx.</t>
-  </si>
-  <si>
-    <t>Trục phản biện</t>
+    <t xml:space="preserve">Thay đổi từ v1 → v2 sau tự rà soát</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhóm không có nhóm đối ứng ở chặng kiểm tra chéo, nên các thay đổi dưới đây đến từ việc nhóm tự rà soát bản v1 theo 4 trục (Phạm vi · Framework · Chỉ số · Hành động). Đối chiếu với v1/dashboard_hanh_dong_v1.xlsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trục rà soát</t>
   </si>
   <si>
     <t>v1</t>
@@ -1156,9 +1156,6 @@
     <t>Lý do</t>
   </si>
   <si>
-    <t>Góp ý từ</t>
-  </si>
-  <si>
     <t>TĐ1</t>
   </si>
   <si>
@@ -1171,9 +1168,6 @@
     <t>Đây là activity metric: tăng cả khi AI trả lời sai, và đẩy hệ thống trả lời cả câu lẽ ra phải chuyển người.</t>
   </si>
   <si>
-    <t>Minh hoạ: tự rà soát theo trục Chỉ số (Nguyễn Quang Huy)</t>
-  </si>
-  <si>
     <t>TĐ2</t>
   </si>
   <si>
@@ -1189,9 +1183,6 @@
     <t>Baseline v1 gây hiểu lầm: chỉ trả lời 11/20 câu, judge cùng họ Gemini, không phải dữ liệu thật.</t>
   </si>
   <si>
-    <t>Minh hoạ: tự rà soát theo trục Chỉ số – bằng chứng (Lê Thị Hoài Thương)</t>
-  </si>
-  <si>
     <t>TĐ3</t>
   </si>
   <si>
@@ -1207,9 +1198,6 @@
     <t>Chẩn đoán Gartner-Lite ra 'Dữ liệu THIẾU' nhưng dashboard v1 không đo → framework chỉ để dán nhãn.</t>
   </si>
   <si>
-    <t>Minh hoạ: tự rà soát theo trục Framework (Nguyễn Thị Minh Khánh)</t>
-  </si>
-  <si>
     <t>TĐ4</t>
   </si>
   <si>
@@ -1225,9 +1213,6 @@
     <t>Không ai biết phải làm gì và ai làm khi chỉ số xấu.</t>
   </si>
   <si>
-    <t>Minh hoạ: tự rà soát theo trục Hành động (Đỗ Lê Việt Anh)</t>
-  </si>
-  <si>
     <t>TĐ5</t>
   </si>
   <si>
@@ -1243,9 +1228,6 @@
     <t>Roadmap không phải cổng quyết định.</t>
   </si>
   <si>
-    <t>Minh hoạ: tự rà soát theo trục Hành động – lộ trình (Lê Thị Châm Anh)</t>
-  </si>
-  <si>
     <t>TĐ6</t>
   </si>
   <si>
@@ -1259,9 +1241,6 @@
   </si>
   <si>
     <t>Tỷ lệ nộp hồ sơ phụ thuộc mùa vụ, không quy được cho AI; CSAT là tự khai, tỷ lệ phản hồi thấp.</t>
-  </si>
-  <si>
-    <t>Minh hoạ: tự rà soát theo trục Chỉ số – giá trị (Lại Bá Quân)</t>
   </si>
   <si>
     <t>Tự kiểm theo yêu cầu nộp bài (§6.4) — tính bằng công thức từ sheet Dashboard</t>
@@ -3314,7 +3293,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3322,20 +3301,19 @@
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="50" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
@@ -3351,128 +3329,107 @@
       <c r="E4" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="F4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>359</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>360</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>221</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="E5" s="4" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="B6" s="4" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="D6" s="4" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="B7" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="C7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="B8" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="B8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>378</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>380</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+    <row r="10" spans="1:5" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>384</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>387</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>389</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>391</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>392</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -3491,23 +3448,23 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>65</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="B4" s="10">
         <f>COUNTIF(Dashboard!$B$5:$B$16,"Product")</f>
@@ -3519,7 +3476,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTIF(Dashboard!$B$5:$B$16,"Workflow")</f>
@@ -3531,79 +3488,79 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B6" s="10">
         <f>COUNTBLANK(Dashboard!$G$5:$G$16)</f>
         <v>0</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTBLANK(Dashboard!$H$5:$H$16)</f>
         <v>0</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="B8" s="10">
         <f>COUNTBLANK(Dashboard!$I$5:$I$16)</f>
         <v>0</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="B9" s="10">
         <f>COUNTBLANK(Dashboard!$K$5:$K$16)</f>
         <v>0</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B10" s="10">
         <f>COUNTBLANK(Dashboard!$M$5:$M$16)</f>
         <v>0</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="B11" s="10">
         <f>COUNTIF(Dashboard!$D$5:$D$16,"3*")+COUNTIF(Dashboard!$D$5:$D$16,"4*")+COUNTIF(Dashboard!$D$5:$D$16,"5*")</f>
         <v>11</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="B12" s="10">
         <f>COUNTIF(Dashboard!$N$5:$N$16,"Quyết định")</f>

</xml_diff>